<commit_message>
update code with latest ggplot2; uses right imports
</commit_message>
<xml_diff>
--- a/inst/extdata/ex01/User_06062018.xlsx
+++ b/inst/extdata/ex01/User_06062018.xlsx
@@ -5,11 +5,11 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Profils\mcanouil\Downloads\DATA\endoc_beta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Profils\mcanouil\Downloads\DATA\endoc_beta\ex01\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11400"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Blank" sheetId="3" r:id="rId1"/>
@@ -49,12 +49,6 @@
     <t>BLANK</t>
   </si>
   <si>
-    <t>SN1</t>
-  </si>
-  <si>
-    <t>SN2</t>
-  </si>
-  <si>
     <t>Sample</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
   </si>
   <si>
     <t>Concentration (µg/L)</t>
-  </si>
-  <si>
-    <t>LYSAT</t>
   </si>
   <si>
     <t>Target</t>
@@ -134,6 +125,15 @@
   </si>
   <si>
     <t>0.5 mM Glc + A</t>
+  </si>
+  <si>
+    <t>LYSATE</t>
+  </si>
+  <si>
+    <t>SUPERNATANT1</t>
+  </si>
+  <si>
+    <t>SUPERNATANT2</t>
   </si>
 </sst>
 </file>
@@ -233,7 +233,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -460,7 +459,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -578,7 +576,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2923,13 +2920,13 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>1</v>
@@ -2938,19 +2935,19 @@
         <v>0</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="N1" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -2958,10 +2955,10 @@
         <v>43257</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>4</v>
@@ -3212,22 +3209,22 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>1</v>
@@ -3236,19 +3233,19 @@
         <v>0</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -3269,16 +3266,16 @@
         <v>siNTP</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I2" s="1">
         <v>0.9048581</v>
@@ -3321,16 +3318,16 @@
         <v>siNTP</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I3" s="1">
         <v>0.84551410000000005</v>
@@ -3373,16 +3370,16 @@
         <v>siNTP</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H4" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I4" s="1">
         <v>0.47709410000000002</v>
@@ -3425,16 +3422,16 @@
         <v>siNTP</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I5" s="1">
         <v>0.32545099999999999</v>
@@ -3477,16 +3474,16 @@
         <v>siNTP</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I6" s="1">
         <v>0.41799199999999997</v>
@@ -3529,16 +3526,16 @@
         <v>siNTP</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I7" s="1">
         <v>0.4046631</v>
@@ -3581,16 +3578,16 @@
         <v>siNTP</v>
       </c>
       <c r="E8" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I8">
         <v>0.3388717</v>
@@ -3635,16 +3632,16 @@
         <v>siNTP</v>
       </c>
       <c r="E9" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I9">
         <v>0.35027330000000001</v>
@@ -3689,16 +3686,16 @@
         <v>siNTP</v>
       </c>
       <c r="E10" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I10">
         <v>0.36398799999999998</v>
@@ -3743,16 +3740,16 @@
         <v>siNTP</v>
       </c>
       <c r="E11" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I11">
         <v>0.30241410000000002</v>
@@ -3797,16 +3794,16 @@
         <v>siNTP</v>
       </c>
       <c r="E12" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I12">
         <v>0.29688639999999999</v>
@@ -3851,16 +3848,16 @@
         <v>siNTP</v>
       </c>
       <c r="E13" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I13">
         <v>0.31960640000000001</v>
@@ -3905,16 +3902,16 @@
         <v>siNTP</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H14" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I14" s="1">
         <v>0.3299955</v>
@@ -3959,16 +3956,16 @@
         <v>siNTP</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H15" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I15" s="1">
         <v>0.26299479999999997</v>
@@ -4013,16 +4010,16 @@
         <v>siNTP</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="H16" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I16" s="1">
         <v>0.32744040000000002</v>
@@ -4067,16 +4064,16 @@
         <v>siNTP</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I17" s="1">
         <v>0.82464230000000005</v>
@@ -4121,16 +4118,16 @@
         <v>siNTP</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I18" s="1">
         <v>0.78054979999999996</v>
@@ -4175,16 +4172,16 @@
         <v>siNTP</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I19" s="1">
         <v>1.05976</v>
@@ -4243,22 +4240,22 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>1</v>
@@ -4267,19 +4264,19 @@
         <v>0</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -4300,16 +4297,16 @@
         <v>siGENE</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I2" s="1">
         <v>0.27928570000000003</v>
@@ -4352,16 +4349,16 @@
         <v>siGENE</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I3" s="1">
         <v>0.59304579999999996</v>
@@ -4404,16 +4401,16 @@
         <v>siGENE</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I4" s="1">
         <v>0.2982032</v>
@@ -4456,16 +4453,16 @@
         <v>siGENE</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I5" s="1">
         <v>0.2879813</v>
@@ -4508,16 +4505,16 @@
         <v>siGENE</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I6" s="1">
         <v>0.267654</v>
@@ -4560,16 +4557,16 @@
         <v>siGENE</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I7" s="1">
         <v>0.33135920000000002</v>
@@ -4612,16 +4609,16 @@
         <v>siGENE</v>
       </c>
       <c r="E8" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I8">
         <v>0.263797</v>
@@ -4666,16 +4663,16 @@
         <v>siGENE</v>
       </c>
       <c r="E9" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I9">
         <v>0.22956480000000001</v>
@@ -4720,16 +4717,16 @@
         <v>siGENE</v>
       </c>
       <c r="E10" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I10">
         <v>0.23144609999999999</v>
@@ -4774,16 +4771,16 @@
         <v>siGENE</v>
       </c>
       <c r="E11" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I11">
         <v>0.37287310000000001</v>
@@ -4828,16 +4825,16 @@
         <v>siGENE</v>
       </c>
       <c r="E12" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I12">
         <v>0.37397249999999999</v>
@@ -4882,16 +4879,16 @@
         <v>siGENE</v>
       </c>
       <c r="E13" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I13">
         <v>0.3727896</v>
@@ -4936,16 +4933,16 @@
         <v>siGENE</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I14" s="1">
         <v>0.31245030000000001</v>
@@ -4990,16 +4987,16 @@
         <v>siGENE</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I15" s="1">
         <v>0.2587759</v>
@@ -5044,16 +5041,16 @@
         <v>siGENE</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="I16" s="1">
         <v>0.26214890000000002</v>
@@ -5098,16 +5095,16 @@
         <v>siGENE</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I17" s="1">
         <v>0.60261849999999995</v>
@@ -5152,16 +5149,16 @@
         <v>siGENE</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I18" s="1">
         <v>0.50985760000000002</v>
@@ -5206,16 +5203,16 @@
         <v>siGENE</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I19" s="1">
         <v>0.69784299999999999</v>

</xml_diff>